<commit_message>
adjusted rule to focus on the suppdm requirement check as neighbor rules focus on counts
</commit_message>
<xml_diff>
--- a/rules/CORE-000844/negative/01/data/unit-test-coreid-CG0531-negative.xlsx
+++ b/rules/CORE-000844/negative/01/data/unit-test-coreid-CG0531-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\verisian\core-contributor\rules\CORE-000844\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0EB55D-C387-4E52-9502-3590C51A3F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB78816F-6A0A-4B83-B97D-CB300F386568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29475" yWindow="1350" windowWidth="26790" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="94">
   <si>
     <t>Product</t>
   </si>
@@ -304,10 +304,7 @@
     <t>Record</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>$multiple_race</t>
+    <t>ASIAN</t>
   </si>
 </sst>
 </file>
@@ -333,7 +330,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -344,6 +341,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -374,7 +377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -385,6 +388,9 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -746,6 +752,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -777,14 +791,14 @@
       <c r="C2" t="s">
         <v>92</v>
       </c>
-      <c r="D2" t="s">
-        <v>93</v>
+      <c r="D2">
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1124,7 +1138,7 @@
       <c r="B5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>70</v>
       </c>
       <c r="D5" s="5" t="s">
@@ -1165,8 +1179,8 @@
       <c r="Q5" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R5" s="6" t="s">
-        <v>80</v>
+      <c r="R5" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="S5" s="5" t="s">
         <v>81</v>
@@ -1196,7 +1210,7 @@
       <c r="B6" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>86</v>
       </c>
       <c r="D6" s="5" t="s">

</xml_diff>